<commit_message>
Sync website and evidence files to WebDeploy
</commit_message>
<xml_diff>
--- a/WebDeploy/Eviden_aunqa68/หลักฐานสายสนับสนุน/AUNQA_extracted_-_ค่า_FTES_ปีการศึกษา_2567_[11_6_2568].xlsx
+++ b/WebDeploy/Eviden_aunqa68/หลักฐานสายสนับสนุน/AUNQA_extracted_-_ค่า_FTES_ปีการศึกษา_2567_[11_6_2568].xlsx
@@ -2208,13 +2208,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93183E7F-D57D-4A87-9E4A-86ED47584CCE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEA39AF9-7845-482C-911A-31CD52106949}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63D2B0FB-56C0-4EF7-9C29-92D9E5F50CF1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6EAA5AC3-727A-446E-987E-D590FCC2D81C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{823DD978-EA75-4E16-A5F8-74CAC87E8BFE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AAB191F-AF22-495E-BB40-989887505F74}"/>
 </file>
</xml_diff>